<commit_message>
add retention cleanup for trade doc imports
</commit_message>
<xml_diff>
--- a/conciliacionpro-frontend/public/templates/Plantilla_carga_masiva_documentos_tributarios.xlsx
+++ b/conciliacionpro-frontend/public/templates/Plantilla_carga_masiva_documentos_tributarios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\orlando.paredes\Documents\Conciliador\conciliacionpro-frontend\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{39103EEE-E9DE-4A82-9DC0-CD817C126651}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EA3B3AD-B273-4196-9B0D-ACF60D19D1AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,12 +23,11 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">LINEAS!$A$1:$L$1</definedName>
   </definedNames>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="138">
   <si>
     <t>Amarillo claro = campo obligatorio</t>
   </si>
@@ -421,6 +420,27 @@
   </si>
   <si>
     <t>Comision Payment</t>
+  </si>
+  <si>
+    <t>2026-04-03</t>
+  </si>
+  <si>
+    <t>2026-04-04</t>
+  </si>
+  <si>
+    <t>2026-04-05</t>
+  </si>
+  <si>
+    <t>2026-04-06</t>
+  </si>
+  <si>
+    <t>2026-04-07</t>
+  </si>
+  <si>
+    <t>0201020</t>
+  </si>
+  <si>
+    <t>01020500</t>
   </si>
 </sst>
 </file>
@@ -430,7 +450,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -468,6 +488,10 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Carlito"/>
     </font>
   </fonts>
@@ -563,7 +587,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -603,18 +627,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -652,21 +664,27 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="21">
-    <dxf>
-      <font>
-        <color rgb="FFB91C1C"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFECACA"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="18">
     <dxf>
       <font>
         <color rgb="FFB91C1C"/>
@@ -756,14 +774,6 @@
       </fill>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
       <fill>
         <patternFill patternType="solid">
@@ -797,32 +807,10 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="FFB91C1C"/>
-      </font>
       <fill>
-        <patternFill>
-          <bgColor rgb="FFFECACA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFB91C1C"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFECACA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFB91C1C"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFECACA"/>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFE2F0D9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -846,6 +834,9 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
       <font>
@@ -873,7 +864,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="DocsTemplate" displayName="DocsTemplate" ref="A1:L11" headerRowDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="DocsTemplate" displayName="DocsTemplate" ref="A1:L11" headerRowDxfId="17">
   <autoFilter ref="A1:L11" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="fiscal_doc_code"/>
@@ -882,7 +873,7 @@
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="issue_date"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="due_date"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="currency_code"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="branch_code"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="branch_code" dataDxfId="16"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="counterparty_identifier"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="counterparty_name"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="reference"/>
@@ -894,19 +885,19 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="PaymentsTemplate" displayName="PaymentsTemplate" ref="A1:J8" headerRowDxfId="19" dataDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="PaymentsTemplate" displayName="PaymentsTemplate" ref="A1:J8" headerRowDxfId="15" dataDxfId="14">
   <autoFilter ref="A1:J8" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="fiscal_doc_code" dataDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="number" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="payment_no" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="payment_date" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="method" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="amount" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="reference" dataDxfId="9"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="card_kind" dataDxfId="8"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="card_last4" dataDxfId="7"/>
-    <tableColumn id="10" xr3:uid="{0534BF47-D54D-4774-8D94-5F2735B5E6BF}" name="auth_code" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="fiscal_doc_code" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="number" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="payment_no" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="payment_date" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="method" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="amount" dataDxfId="8"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="reference" dataDxfId="7"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="card_kind" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0100-000009000000}" name="card_last4" dataDxfId="5"/>
+    <tableColumn id="10" xr3:uid="{0534BF47-D54D-4774-8D94-5F2735B5E6BF}" name="auth_code" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1069,14 +1060,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="17.399999999999999">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="33" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="1"/>
@@ -1087,14 +1078,14 @@
       <c r="F2" s="1"/>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="B3" s="17"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
+      <c r="B3" s="32"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="2" t="s">
@@ -1115,14 +1106,14 @@
       <c r="F5" s="1"/>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="32" t="s">
         <v>74</v>
       </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="17"/>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
+      <c r="B6" s="32"/>
+      <c r="C6" s="32"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="32"/>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="2" t="s">
@@ -1203,14 +1194,14 @@
       <c r="F14" s="1"/>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="17" t="s">
+      <c r="A15" s="32" t="s">
         <v>82</v>
       </c>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="17"/>
+      <c r="B15" s="32"/>
+      <c r="C15" s="32"/>
+      <c r="D15" s="32"/>
+      <c r="E15" s="32"/>
+      <c r="F15" s="32"/>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="2" t="s">
@@ -1261,14 +1252,14 @@
       <c r="F20" s="1"/>
     </row>
     <row r="21" spans="1:6">
-      <c r="A21" s="17" t="s">
+      <c r="A21" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="B21" s="17"/>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17"/>
+      <c r="B21" s="32"/>
+      <c r="C21" s="32"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="32"/>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="2" t="s">
@@ -1289,14 +1280,14 @@
       <c r="F23" s="1"/>
     </row>
     <row r="24" spans="1:6">
-      <c r="A24" s="17" t="s">
+      <c r="A24" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="B24" s="17"/>
-      <c r="C24" s="17"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="17"/>
-      <c r="F24" s="17"/>
+      <c r="B24" s="32"/>
+      <c r="C24" s="32"/>
+      <c r="D24" s="32"/>
+      <c r="E24" s="32"/>
+      <c r="F24" s="32"/>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="2" t="s">
@@ -1367,14 +1358,14 @@
       <c r="F31" s="1"/>
     </row>
     <row r="32" spans="1:6">
-      <c r="A32" s="17" t="s">
+      <c r="A32" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="B32" s="17"/>
-      <c r="C32" s="17"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="17"/>
-      <c r="F32" s="17"/>
+      <c r="B32" s="32"/>
+      <c r="C32" s="32"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="32"/>
+      <c r="F32" s="32"/>
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="2" t="s">
@@ -1405,14 +1396,14 @@
       <c r="F35" s="1"/>
     </row>
     <row r="36" spans="1:6">
-      <c r="A36" s="17" t="s">
+      <c r="A36" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="B36" s="17"/>
-      <c r="C36" s="17"/>
-      <c r="D36" s="17"/>
-      <c r="E36" s="17"/>
-      <c r="F36" s="17"/>
+      <c r="B36" s="32"/>
+      <c r="C36" s="32"/>
+      <c r="D36" s="32"/>
+      <c r="E36" s="32"/>
+      <c r="F36" s="32"/>
     </row>
     <row r="37" spans="1:6">
       <c r="A37" s="2" t="s">
@@ -1509,10 +1500,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="16.8">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="34" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="20"/>
+      <c r="B1" s="35"/>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="10"/>
@@ -1690,7 +1681,7 @@
     <col min="1" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
     <col min="4" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="7" max="7" width="16" style="31" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
     <col min="9" max="9" width="28" customWidth="1"/>
     <col min="10" max="10" width="24.5" bestFit="1" customWidth="1"/>
@@ -1698,41 +1689,41 @@
     <col min="12" max="12" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="21" customFormat="1" ht="27.6">
-      <c r="A1" s="22" t="s">
+    <row r="1" spans="1:12" s="17" customFormat="1" ht="27.6">
+      <c r="A1" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="23" t="s">
+      <c r="C1" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="24" t="s">
+      <c r="D1" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="24" t="s">
+      <c r="E1" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="F1" s="23" t="s">
+      <c r="F1" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="G1" s="23" t="s">
+      <c r="G1" s="30" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="23" t="s">
+      <c r="H1" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="23" t="s">
+      <c r="I1" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="25" t="s">
+      <c r="J1" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="K1" s="25" t="s">
+      <c r="K1" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="L1" s="26" t="s">
+      <c r="L1" s="22" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1755,8 +1746,8 @@
       <c r="F2" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="G2" s="3">
-        <v>201020</v>
+      <c r="G2" s="16" t="s">
+        <v>136</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>89</v>
@@ -1789,8 +1780,8 @@
       <c r="F3" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="G3" s="3">
-        <v>1020500</v>
+      <c r="G3" s="16" t="s">
+        <v>137</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>92</v>
@@ -1823,8 +1814,8 @@
       <c r="F4" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="G4" s="3">
-        <v>201020</v>
+      <c r="G4" s="16" t="s">
+        <v>136</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>95</v>
@@ -1857,8 +1848,8 @@
       <c r="F5" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="G5" s="3">
-        <v>1020500</v>
+      <c r="G5" s="16" t="s">
+        <v>137</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>98</v>
@@ -1891,8 +1882,8 @@
       <c r="F6" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="3">
-        <v>201020</v>
+      <c r="G6" s="16" t="s">
+        <v>136</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>101</v>
@@ -1925,8 +1916,8 @@
       <c r="F7" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="G7" s="3">
-        <v>1020500</v>
+      <c r="G7" s="16" t="s">
+        <v>137</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>104</v>
@@ -1959,8 +1950,8 @@
       <c r="F8" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="G8" s="3">
-        <v>201020</v>
+      <c r="G8" s="16" t="s">
+        <v>136</v>
       </c>
       <c r="H8" s="3" t="s">
         <v>107</v>
@@ -1993,8 +1984,8 @@
       <c r="F9" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="G9" s="3">
-        <v>1020500</v>
+      <c r="G9" s="16" t="s">
+        <v>137</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>92</v>
@@ -2031,8 +2022,8 @@
       <c r="F10" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="G10" s="3">
-        <v>201020</v>
+      <c r="G10" s="16" t="s">
+        <v>136</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>95</v>
@@ -2069,8 +2060,8 @@
       <c r="F11" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="G11" s="3">
-        <v>201020</v>
+      <c r="G11" s="16" t="s">
+        <v>136</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>95</v>
@@ -2082,10 +2073,10 @@
         <v>112</v>
       </c>
       <c r="K11" s="3">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="L11" s="7">
-        <v>5003</v>
+        <v>6002</v>
       </c>
     </row>
   </sheetData>
@@ -2123,41 +2114,41 @@
     <col min="10" max="12" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="27" customFormat="1" ht="27.6">
-      <c r="A1" s="22" t="s">
+    <row r="1" spans="1:12" s="23" customFormat="1" ht="27.6">
+      <c r="A1" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="B1" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="23" t="s">
+      <c r="C1" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="D1" s="23" t="s">
+      <c r="D1" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="E1" s="25" t="s">
+      <c r="E1" s="21" t="s">
         <v>37</v>
       </c>
-      <c r="F1" s="23" t="s">
+      <c r="F1" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="G1" s="23" t="s">
+      <c r="G1" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="H1" s="23" t="s">
+      <c r="H1" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="I1" s="25" t="s">
+      <c r="I1" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="J1" s="23" t="s">
+      <c r="J1" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="K1" s="23" t="s">
+      <c r="K1" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="L1" s="25" t="s">
+      <c r="L1" s="21" t="s">
         <v>44</v>
       </c>
     </row>
@@ -2703,18 +2694,18 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:L1" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
+  <conditionalFormatting sqref="E1">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="I1:I16">
-    <cfRule type="cellIs" dxfId="4" priority="3" operator="lessThan">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L1">
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E1">
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2737,35 +2728,35 @@
     <col min="9" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="33" customFormat="1">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:10" s="29" customFormat="1">
+      <c r="A1" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="29" t="s">
+      <c r="B1" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="29" t="s">
+      <c r="C1" s="25" t="s">
         <v>83</v>
       </c>
-      <c r="D1" s="30" t="s">
+      <c r="D1" s="26" t="s">
         <v>84</v>
       </c>
-      <c r="E1" s="29" t="s">
+      <c r="E1" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="F1" s="29" t="s">
+      <c r="F1" s="25" t="s">
         <v>86</v>
       </c>
-      <c r="G1" s="31" t="s">
+      <c r="G1" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="H1" s="31" t="s">
+      <c r="H1" s="27" t="s">
         <v>64</v>
       </c>
-      <c r="I1" s="32" t="s">
+      <c r="I1" s="28" t="s">
         <v>87</v>
       </c>
-      <c r="J1" s="32" t="s">
+      <c r="J1" s="28" t="s">
         <v>88</v>
       </c>
     </row>
@@ -2831,8 +2822,8 @@
       <c r="C4" s="3">
         <v>1</v>
       </c>
-      <c r="D4" s="16">
-        <v>46115</v>
+      <c r="D4" s="16" t="s">
+        <v>131</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>56</v>
@@ -2857,8 +2848,8 @@
       <c r="C5" s="3">
         <v>2</v>
       </c>
-      <c r="D5" s="16">
-        <v>46115</v>
+      <c r="D5" s="16" t="s">
+        <v>132</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>58</v>
@@ -2889,8 +2880,8 @@
       <c r="C6" s="3">
         <v>1</v>
       </c>
-      <c r="D6" s="16">
-        <v>46116</v>
+      <c r="D6" s="16" t="s">
+        <v>133</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>60</v>
@@ -2915,8 +2906,8 @@
       <c r="C7" s="3">
         <v>2</v>
       </c>
-      <c r="D7" s="16">
-        <v>46116</v>
+      <c r="D7" s="16" t="s">
+        <v>134</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>58</v>
@@ -2947,8 +2938,8 @@
       <c r="C8" s="3">
         <v>1</v>
       </c>
-      <c r="D8" s="16">
-        <v>46118</v>
+      <c r="D8" s="16" t="s">
+        <v>135</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>60</v>
@@ -2964,11 +2955,9 @@
       <c r="J8" s="7"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="7" type="noConversion"/>
   <conditionalFormatting sqref="F1">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThanOrEqual">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="lessThanOrEqual">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>